<commit_message>
pinterest: şablonun yönlendirme satırı boşaltıldı (içe aktarma 60 OK, 1 ERROR)
İçe aktarma hata raporu: 60 pin satırının hepsi OK; tek ERROR şablonun
2. satırındaki yönlendirme metniydi ("Enter image URL (required)" …).
Satır silinmedi, boşaltıldı (J sütunundaki STATUS formülleri satır
referanslı). openpyxl cell(value=None) atamayı atladığı için doğrudan
.value = None kullanıldı; dosya geri okunarak doğrulandı: satır 2 boş,
60 pin satır 3 ila 62, açılır listeler korunuyor. second-brain dersi eklendi.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0155ChXCESvn4jMw6J2DsxxU
</commit_message>
<xml_diff>
--- a/docs/artifact-studio/pinterest/artifact-studio-pinterest-60.xlsx
+++ b/docs/artifact-studio/pinterest/artifact-studio-pinterest-60.xlsx
@@ -528,56 +528,16 @@
       </c>
     </row>
     <row r="2" customFormat="1" s="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Enter image URL (required)</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Pin title (optional, max 100)</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Description (optional, max 500)</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Alt text (optional, max 500)</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Destination URL (optional)</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Select from dropdown (required)</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Section (optional)</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Select: low/medium/high</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Select ratio</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Auto-validated</t>
-        </is>
-      </c>
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">

</xml_diff>